<commit_message>
P2 y P3: salud del cronograma y Monte Carlo del plazo
Chequeo de salud con semáforo (diez comprobaciones al estilo DCMA-14; el
rojo bloquea la simulación). Monte Carlo del plazo vectorizado por
bloques, con duraciones PERT (algoritmo de Cheng) o triangulares y
riesgos de plazo al estilo AACE 57R-09 desde la hoja «Riesgos de plazo»:
P50/P80/P90, probabilidad de cumplir el cronograma, curva S, criticidad,
días de P80 por riesgo y resumen en palabras. Hoja «Cronograma
(simulación)» con gráfico y Gantt probabilístico.

Libro de pruebas ampliado (riesgos, salud y Monte Carlo de referencia en
Python), bloque Q11–Q20 de la guía, benchmark y hojas reales en el banco.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -11,6 +11,9 @@
     <sheet name="Actividades" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Calendario" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Esperado" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Riesgos de plazo" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Esperado (salud)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Esperado (simulación)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +90,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -523,60 +527,74 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>«Riesgos de plazo»: cinco riesgos (uno es una oportunidad) que alargan a la vez sus actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>«Esperado»: las fechas que debe dar el complemento, calculadas aparte por el script.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>«Esperado (salud)» y «Esperado (simulación)»: el semáforo y el Monte Carlo de referencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Cómo se usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>bloque Q (docs/GUIA_PRUEBAS_EXCEL.md).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Resultado esperado, en una línea</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Fin del proyecto: 16/07/2027 · 118 días laborables · 12 actividades críticas.</t>
         </is>
@@ -2357,4 +2375,784 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Riesgos de plazo — cada uno alarga a la vez todas sus actividades (AACE 57R-09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Riesgo</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Probabilidad</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto mínimo</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto más probable</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto máximo</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Actividades afectadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lluvias intensas durante la obra gris</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Obra gris</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Demora en la licencia de construcción</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Retraso del proveedor del ascensor</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bajo rendimiento de la cuadrilla de acabados</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Acabados</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Oportunidad: estructura prefabricada</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Chequeo de salud esperado (calculado por el script)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Comprobación</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Semáforo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>logica</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>adelantos</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>retardos</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>relaciones</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>restricciones</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>holgura-negativa</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>holgura-alta</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>duracion-larga</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>amarillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>incertidumbre</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>convergencias</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Monte Carlo de referencia: 20000 iteraciones en Python (PERT + riesgos de plazo). El complemento usa otros números aleatorios: debe coincidir en ±1 día y ±3 puntos de criticidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Percentil</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Días laborables</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Fecha de fin</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>124</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>46595</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>135</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>46610</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P80</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>143</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>46623</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>148</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>46630</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Índice de criticidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Inicio del proyecto</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>0.993</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Permisos y licencias</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>0.735</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Diseño detallado</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>0.259</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Movilización de obra</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>0.735</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Excavación</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>0.993</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Cimentación</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>0.993</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Estructura</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>0.993</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Fabricación del ascensor</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Cubierta</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>0.115</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Instalaciones hidráulicas</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Mampostería</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>0.878</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Montaje del ascensor</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Acabados interiores</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>0.878</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Fachada</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>0.115</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Pruebas de instalaciones</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Paisajismo</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Limpieza final</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Entrega al cliente</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Vigilancia hasta la entrega</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
P1: avance real (fecha de corte, fechas reales, % completado, restante) y restricciones de fin
Las mismas reglas en el CPM y en la simulación (red.ts): terminadas
fijas, en curso desde la fecha de corte con lo que queda, pendientes no
antes del corte; «no después de» limita las fechas tardías. Columna
Estado, gris y línea de corte en el Gantt, salud con restricciones duras.
Escenario con avance en el libro de pruebas, calculado aparte en Python.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -14,6 +14,8 @@
     <sheet name="Riesgos de plazo" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Esperado (salud)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Esperado (simulación)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Avance (prueba)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Esperado (con avance)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -89,8 +91,8 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -546,55 +548,69 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>«Avance (prueba)» y «Esperado (con avance)»: un escenario con fecha de corte, fechas reales,</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>% completado, duración restante y restricciones de fin, con su resultado esperado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Cómo se usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>bloque Q (docs/GUIA_PRUEBAS_EXCEL.md).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Resultado esperado, en una línea</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Fin del proyecto: 16/07/2027 · 118 días laborables · 12 actividades críticas.</t>
         </is>
@@ -611,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -624,6 +640,13 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -684,6 +707,41 @@
           <t>Inicio no antes de</t>
         </is>
       </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Inicio real</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Fin real</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>% completado</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Duración restante</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Inicio no después de</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Terminar no antes de</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Terminar no después de</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -708,6 +766,12 @@
       <c r="I4" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="n"/>
+      <c r="M4" s="7" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
+      <c r="Q4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -745,6 +809,12 @@
       <c r="I5" s="5" t="n">
         <v>200</v>
       </c>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="n"/>
+      <c r="M5" s="7" t="n"/>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="6" t="n"/>
+      <c r="Q5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -782,6 +852,12 @@
       <c r="I6" s="5" t="n">
         <v>900</v>
       </c>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
+      <c r="Q6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -819,6 +895,12 @@
       <c r="I7" s="5" t="n">
         <v>1500</v>
       </c>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
+      <c r="Q7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -856,6 +938,12 @@
       <c r="I8" s="5" t="n">
         <v>2500</v>
       </c>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
+      <c r="Q8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -893,6 +981,12 @@
       <c r="I9" s="5" t="n">
         <v>3000</v>
       </c>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
+      <c r="M9" s="7" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
+      <c r="Q9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -930,6 +1024,12 @@
       <c r="I10" s="5" t="n">
         <v>3500</v>
       </c>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="7" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
+      <c r="Q10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -967,6 +1067,12 @@
       <c r="I11" s="5" t="n">
         <v>100</v>
       </c>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="7" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
+      <c r="Q11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1004,6 +1110,12 @@
       <c r="I12" s="5" t="n">
         <v>2200</v>
       </c>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+      <c r="M12" s="7" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
+      <c r="Q12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1041,6 +1153,12 @@
       <c r="I13" s="5" t="n">
         <v>1800</v>
       </c>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+      <c r="M13" s="7" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
+      <c r="Q13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1078,6 +1196,12 @@
       <c r="I14" s="5" t="n">
         <v>1600</v>
       </c>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="7" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
+      <c r="Q14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1115,6 +1239,12 @@
       <c r="I15" s="5" t="n">
         <v>2000</v>
       </c>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="M15" s="7" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="n"/>
+      <c r="Q15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1152,6 +1282,12 @@
       <c r="I16" s="5" t="n">
         <v>1200</v>
       </c>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="M16" s="7" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
+      <c r="Q16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1189,6 +1325,12 @@
       <c r="I17" s="5" t="n">
         <v>2400</v>
       </c>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="7" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
+      <c r="Q17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1226,6 +1368,12 @@
       <c r="I18" s="5" t="n">
         <v>1900</v>
       </c>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="M18" s="7" t="n"/>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
+      <c r="Q18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1263,6 +1411,12 @@
       <c r="I19" s="5" t="n">
         <v>800</v>
       </c>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="M19" s="7" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
+      <c r="Q19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1303,6 +1457,12 @@
       <c r="J20" s="6" t="n">
         <v>46566</v>
       </c>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+      <c r="M20" s="7" t="n"/>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6" t="n"/>
+      <c r="Q20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1340,6 +1500,12 @@
       <c r="I21" s="5" t="n">
         <v>500</v>
       </c>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+      <c r="M21" s="7" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="n"/>
+      <c r="Q21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1368,6 +1534,12 @@
       <c r="I22" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+      <c r="M22" s="7" t="n"/>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6" t="n"/>
+      <c r="Q22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1396,6 +1568,12 @@
       <c r="I23" s="5" t="n">
         <v>150</v>
       </c>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+      <c r="M23" s="7" t="n"/>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="n"/>
+      <c r="Q23" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1408,7 +1586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1423,6 +1601,19 @@
       </c>
       <c r="B1" s="6" t="n">
         <v>46419</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fecha de corte</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>(vacía: sin avance; ver «Avance (prueba)»)</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -1584,7 +1775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1596,6 +1787,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1671,6 +1863,11 @@
           <t>Crítica</t>
         </is>
       </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1701,9 +1898,14 @@
       <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1736,9 +1938,14 @@
       <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1771,9 +1978,14 @@
       <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1806,9 +2018,14 @@
       <c r="H9" t="n">
         <v>0</v>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1841,9 +2058,14 @@
       <c r="H10" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1876,9 +2098,14 @@
       <c r="H11" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1911,9 +2138,14 @@
       <c r="H12" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -1951,6 +2183,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1986,6 +2223,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2021,6 +2263,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2056,6 +2303,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2086,9 +2338,14 @@
       <c r="H17" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -2126,6 +2383,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2156,9 +2418,14 @@
       <c r="H19" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -2196,6 +2463,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2231,6 +2503,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2266,6 +2543,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2296,9 +2578,14 @@
       <c r="H23" t="n">
         <v>0</v>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -2331,9 +2618,14 @@
       <c r="H24" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -2366,9 +2658,14 @@
       <c r="H25" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>Sí</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -2450,16 +2747,16 @@
           <t>Lluvias intensas durante la obra gris</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="7" t="n">
         <v>0.05</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -2479,16 +2776,16 @@
           <t>Demora en la licencia de construcción</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -2508,16 +2805,16 @@
           <t>Retraso del proveedor del ascensor</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="7" t="n">
         <v>0.4</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -2537,16 +2834,16 @@
           <t>Bajo rendimiento de la cuadrilla de acabados</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="7" t="n">
         <v>0.25</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="7" t="n">
         <v>0.05</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="7" t="n">
         <v>0.15</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -2566,16 +2863,16 @@
           <t>Oportunidad: estructura prefabricada</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>-0.15</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="7" t="n">
         <v>-0.1</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="7" t="n">
         <v>-0.05</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -2863,7 +3160,7 @@
           <t>Inicio del proyecto</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="7" t="n">
         <v>0.993</v>
       </c>
     </row>
@@ -2878,7 +3175,7 @@
           <t>Permisos y licencias</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>0.735</v>
       </c>
     </row>
@@ -2893,7 +3190,7 @@
           <t>Diseño detallado</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="7" t="n">
         <v>0.259</v>
       </c>
     </row>
@@ -2908,7 +3205,7 @@
           <t>Movilización de obra</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>0.735</v>
       </c>
     </row>
@@ -2923,7 +3220,7 @@
           <t>Excavación</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="7" t="n">
         <v>0.993</v>
       </c>
     </row>
@@ -2938,7 +3235,7 @@
           <t>Cimentación</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="7" t="n">
         <v>0.993</v>
       </c>
     </row>
@@ -2953,7 +3250,7 @@
           <t>Estructura</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="7" t="n">
         <v>0.993</v>
       </c>
     </row>
@@ -2968,7 +3265,7 @@
           <t>Fabricación del ascensor</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2983,7 +3280,7 @@
           <t>Cubierta</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="7" t="n">
         <v>0.115</v>
       </c>
     </row>
@@ -2998,7 +3295,7 @@
           <t>Instalaciones eléctricas</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3013,7 +3310,7 @@
           <t>Instalaciones hidráulicas</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3028,7 +3325,7 @@
           <t>Mampostería</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="7" t="n">
         <v>0.878</v>
       </c>
     </row>
@@ -3043,7 +3340,7 @@
           <t>Montaje del ascensor</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3058,7 +3355,7 @@
           <t>Acabados interiores</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C24" s="7" t="n">
         <v>0.878</v>
       </c>
     </row>
@@ -3073,7 +3370,7 @@
           <t>Fachada</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="7" t="n">
         <v>0.115</v>
       </c>
     </row>
@@ -3088,7 +3385,7 @@
           <t>Pruebas de instalaciones</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3103,7 +3400,7 @@
           <t>Paisajismo</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="7" t="n">
         <v>0.122</v>
       </c>
     </row>
@@ -3118,7 +3415,7 @@
           <t>Limpieza final</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n">
+      <c r="C28" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3133,7 +3430,7 @@
           <t>Entrega al cliente</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n">
+      <c r="C29" s="7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3148,8 +3445,1115 @@
           <t>Vigilancia hasta la entrega</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="7" t="n">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Escenario con avance: copia estos valores en «Actividades» (mismas columnas) y la fecha de corte en «Calendario»!B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fecha de corte</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46461</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Inicio real</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Fin real</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>% completado</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Duración restante</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Terminar no antes de</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Terminar no después de</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="D5" s="7" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="D6" s="7" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="D7" s="7" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>46447</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>46451</v>
+      </c>
+      <c r="D8" s="7" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>46454</v>
+      </c>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>46454</v>
+      </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" t="n">
+        <v>42</v>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n">
+        <v>46568</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="F12" s="6" t="n">
+        <v>46589</v>
+      </c>
+      <c r="G12" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>CPM esperado con el escenario de «Avance (prueba)» (fecha de corte 15/03/2027), calculado por el script</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fin del proyecto</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46595</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Duración (días laborables)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Duración</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Inicio tardío</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Fin tardío</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Holgura total</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inicio del proyecto</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Permisos y licencias</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Diseño detallado</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Movilización de obra</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>46447</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>46451</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>46451</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Terminada</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Excavación</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>46454</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>46468</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>46450</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>46464</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cimentación</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>46469</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>46491</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>46465</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>46489</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Estructura</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>46492</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>46533</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>46490</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>46531</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fabricación del ascensor</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>45</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>46454</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>46520</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>46513</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>46577</v>
+      </c>
+      <c r="H13" t="n">
+        <v>41</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cubierta</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>46534</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>46549</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>46532</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>46547</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>46506</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>46533</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>46527</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>46554</v>
+      </c>
+      <c r="H15" t="n">
+        <v>15</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Instalaciones hidráulicas</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>18</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>46506</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>46531</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>46531</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>46554</v>
+      </c>
+      <c r="H16" t="n">
+        <v>17</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mampostería</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>46527</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>46554</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>46527</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>46554</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Montaje del ascensor</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>46552</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>46561</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>46580</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>46590</v>
+      </c>
+      <c r="H18" t="n">
+        <v>20</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Acabados interiores</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>25</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>46555</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>46590</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>46555</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>46590</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fachada</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>15</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>46552</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>46570</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>46548</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>46568</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pruebas de instalaciones</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>46531</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>46538</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>46590</v>
+      </c>
+      <c r="H21" t="n">
+        <v>37</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paisajismo</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>46575</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>46589</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>46576</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>46590</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Limpieza final</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>46591</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>46591</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Entrega al cliente</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Vigilancia hasta la entrega</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>46581</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>46581</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>46595</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
P5: costo y plazo juntos (JCL) en el módulo Cronograma
Costos fijos, por día, indirectos del proyecto y de los riesgos; el costo
se calcula en la misma iteración que el plazo. Distribución del costo,
probabilidad conjunta (JCL), fecha y presupuesto para un 80 % conjunto,
costo de P80 por riesgo, nube costo–plazo en el panel y en la hoja.
Verificado contra el Monte Carlo de referencia en Python; guía Q36–Q39.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -647,6 +647,7 @@
     <col width="19" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -740,6 +741,11 @@
       <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Terminar no después de</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Costo fijo</t>
         </is>
       </c>
     </row>
@@ -944,6 +950,9 @@
       <c r="O8" s="6" t="n"/>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
+      <c r="R8" s="5" t="n">
+        <v>18000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -987,6 +996,9 @@
       <c r="O9" s="6" t="n"/>
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="6" t="n"/>
+      <c r="R9" s="5" t="n">
+        <v>65000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1030,6 +1042,9 @@
       <c r="O10" s="6" t="n"/>
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
+      <c r="R10" s="5" t="n">
+        <v>140000</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1073,6 +1088,9 @@
       <c r="O11" s="6" t="n"/>
       <c r="P11" s="6" t="n"/>
       <c r="Q11" s="6" t="n"/>
+      <c r="R11" s="5" t="n">
+        <v>95000</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1116,6 +1134,9 @@
       <c r="O12" s="6" t="n"/>
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="6" t="n"/>
+      <c r="R12" s="5" t="n">
+        <v>30000</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1159,6 +1180,9 @@
       <c r="O13" s="6" t="n"/>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
+      <c r="R13" s="5" t="n">
+        <v>42000</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1202,6 +1226,9 @@
       <c r="O14" s="6" t="n"/>
       <c r="P14" s="6" t="n"/>
       <c r="Q14" s="6" t="n"/>
+      <c r="R14" s="5" t="n">
+        <v>36000</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1245,6 +1272,9 @@
       <c r="O15" s="6" t="n"/>
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="6" t="n"/>
+      <c r="R15" s="5" t="n">
+        <v>25000</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1331,6 +1361,9 @@
       <c r="O17" s="6" t="n"/>
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="6" t="n"/>
+      <c r="R17" s="5" t="n">
+        <v>60000</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1374,6 +1407,9 @@
       <c r="O18" s="6" t="n"/>
       <c r="P18" s="6" t="n"/>
       <c r="Q18" s="6" t="n"/>
+      <c r="R18" s="5" t="n">
+        <v>38000</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1463,6 +1499,9 @@
       <c r="O20" s="6" t="n"/>
       <c r="P20" s="6" t="n"/>
       <c r="Q20" s="6" t="n"/>
+      <c r="R20" s="5" t="n">
+        <v>12000</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1705,6 +1744,16 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Costo indirecto por día</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1800</v>
       </c>
     </row>
     <row r="12">
@@ -2680,7 +2729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2690,6 +2739,7 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2735,6 +2785,11 @@
           <t>Actividades afectadas</t>
         </is>
       </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Costo si ocurre</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2793,6 +2848,9 @@
           <t>2</t>
         </is>
       </c>
+      <c r="H5" s="5" t="n">
+        <v>12000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2821,6 +2879,9 @@
         <is>
           <t>8</t>
         </is>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="7">
@@ -3048,18 +3109,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Monte Carlo de referencia: 20000 iteraciones en Python (PERT + riesgos de plazo). El complemento usa otros números aleatorios: debe coincidir en ±1 día y ±3 puntos de criticidad.</t>
+          <t>Monte Carlo de referencia: 20000 iteraciones en Python (PERT + riesgos de plazo). El complemento usa otros números aleatorios: debe coincidir en ±1 día, ±3 puntos de criticidad, ±1 % de costo y ±3 puntos de JCL. El costo determinista es exacto.</t>
         </is>
       </c>
     </row>
@@ -3079,6 +3142,16 @@
           <t>Fecha de fin</t>
         </is>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3092,6 +3165,14 @@
       <c r="C4" s="6" t="n">
         <v>46595</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Determinista (exacto)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1225500</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3105,6 +3186,14 @@
       <c r="C5" s="6" t="n">
         <v>46610</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1256952.34</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3118,6 +3207,14 @@
       <c r="C6" s="6" t="n">
         <v>46623</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1305742.24</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3130,6 +3227,34 @@
       </c>
       <c r="C7" s="6" t="n">
         <v>46630</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>P80</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1343193.94</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>1362802.13</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>JCL: P(plazo ≤ P80 y costo ≤ P80)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0.7597</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
V1: mitigación antes y después
Respuesta, responsable, costo y valores «después» por riesgo; simular
antes, después o comparar con los mismos números aleatorios; por
respuesta, días de P80, ahorro en el P80 del costo y retorno por unidad
invertida; hoja «Cronograma (mitigación)» y resumen en palabras.
Guía Q42–Q44.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -2729,7 +2729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2740,6 +2740,14 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2790,6 +2798,46 @@
           <t>Costo si ocurre</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Costo de la respuesta</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Probabilidad después</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto mínimo después</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto más probable después</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto máximo después</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Costo si ocurre después</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2819,6 +2867,31 @@
           <t>Obra gris</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cubiertas provisionales y bombeo</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Residente de obra</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O4" s="7" t="n">
+        <v>0.12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2851,6 +2924,31 @@
       <c r="H5" s="5" t="n">
         <v>12000</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Contratar un gestor de trámites</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Director del proyecto</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2882,6 +2980,34 @@
       </c>
       <c r="H6" s="5" t="n">
         <v>20000</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pedido con anticipo y penalidad al proveedor</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O6" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
V2: riesgos que añaden trabajo (ramificación probabilística)
Un riesgo puede añadir una actividad (con su duración de tres puntos)
entre unas predecesoras y unas sucesoras; solo existe en las iteraciones
en que ocurre. Pruebas con resultado exacto y guía Q45.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -2729,7 +2729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2748,6 +2748,12 @@
     <col width="24" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2836,6 +2842,36 @@
       <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Costo si ocurre después</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Actividad nueva</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Duración nueva mínima</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Duración nueva más probable</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Duración nueva máxima</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>Después de</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Antes de</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V4: incertidumbre en los costos de cada actividad
- Columnas «Costo fijo mínimo/máximo» y «Costo por día mínimo/máximo» en
  «Actividades»; el costo de su columna es el más probable. La plantilla
  incluye ahora «Costo fijo».
- En la simulación, cada costo con rango se sortea (PERT o triangular)
  con flujos propios: las fechas no cambian. Se mide lo que añade la
  incertidumbre de los costos al P80, en las mismas iteraciones.
- Hoja, resumen en palabras e informe PDF lo cuentan.
- Oráculo Python: «Costos inciertos (prueba)» y «Esperado (costos
  inciertos)»; tests analíticos, de números comunes y en varios hilos.
- Guía Q49–Q50 y documentación al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -16,6 +16,8 @@
     <sheet name="Esperado (simulación)" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Avance (prueba)" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Esperado (con avance)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Costos inciertos (prueba)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Esperado (costos inciertos)" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -562,58 +564,352 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>«Costos inciertos (prueba)» y «Esperado (costos inciertos)»: mínimo y máximo de algunos costos (V4)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>y el Monte Carlo de referencia con ellos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Cómo se usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>bloque Q (docs/GUIA_PRUEBAS_EXCEL.md).</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Resultado esperado, en una línea</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Fin del proyecto: 16/07/2027 · 118 días laborables · 12 actividades críticas.</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>V4: copia estos valores en «Actividades», columnas S a V (mismo ID). El costo fijo y el costo por día de «Actividades» son los más probables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Costo fijo mínimo</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Costo fijo máximo</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Costo por día mínimo</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Costo por día máximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cimentación</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Estructura</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>130000</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>190000</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>4600</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fabricación del ascensor</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Acabados interiores</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>55000</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Monte Carlo de referencia con «Costos inciertos (prueba)»: 20000 iteraciones en Python. Debe coincidir en ±1 % de costo y ±3 puntos de JCL. El plazo no cambia (los costos no mueven fechas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Determinista (exacto; con los más probables)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1225500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1277000.19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1330387.36</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>P80</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1371202.63</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1392794.03</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1333007.23</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>P80 con los costos más probables</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1343453.52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>JCL: P(plazo ≤ P80 y costo ≤ P80)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.7449</v>
       </c>
     </row>
   </sheetData>
@@ -627,7 +923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -648,6 +944,10 @@
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -746,6 +1046,26 @@
       <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Costo fijo</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Costo fijo mínimo</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Costo fijo máximo</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>Costo por día mínimo</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>Costo por día máximo</t>
         </is>
       </c>
     </row>
@@ -778,6 +1098,10 @@
       <c r="O4" s="6" t="n"/>
       <c r="P4" s="6" t="n"/>
       <c r="Q4" s="6" t="n"/>
+      <c r="S4" s="5" t="n"/>
+      <c r="T4" s="5" t="n"/>
+      <c r="U4" s="5" t="n"/>
+      <c r="V4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -821,6 +1145,10 @@
       <c r="O5" s="6" t="n"/>
       <c r="P5" s="6" t="n"/>
       <c r="Q5" s="6" t="n"/>
+      <c r="S5" s="5" t="n"/>
+      <c r="T5" s="5" t="n"/>
+      <c r="U5" s="5" t="n"/>
+      <c r="V5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -864,6 +1192,10 @@
       <c r="O6" s="6" t="n"/>
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="6" t="n"/>
+      <c r="S6" s="5" t="n"/>
+      <c r="T6" s="5" t="n"/>
+      <c r="U6" s="5" t="n"/>
+      <c r="V6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -907,6 +1239,10 @@
       <c r="O7" s="6" t="n"/>
       <c r="P7" s="6" t="n"/>
       <c r="Q7" s="6" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -953,6 +1289,10 @@
       <c r="R8" s="5" t="n">
         <v>18000</v>
       </c>
+      <c r="S8" s="5" t="n"/>
+      <c r="T8" s="5" t="n"/>
+      <c r="U8" s="5" t="n"/>
+      <c r="V8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -999,6 +1339,10 @@
       <c r="R9" s="5" t="n">
         <v>65000</v>
       </c>
+      <c r="S9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="U9" s="5" t="n"/>
+      <c r="V9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1045,6 +1389,10 @@
       <c r="R10" s="5" t="n">
         <v>140000</v>
       </c>
+      <c r="S10" s="5" t="n"/>
+      <c r="T10" s="5" t="n"/>
+      <c r="U10" s="5" t="n"/>
+      <c r="V10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1091,6 +1439,10 @@
       <c r="R11" s="5" t="n">
         <v>95000</v>
       </c>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1137,6 +1489,10 @@
       <c r="R12" s="5" t="n">
         <v>30000</v>
       </c>
+      <c r="S12" s="5" t="n"/>
+      <c r="T12" s="5" t="n"/>
+      <c r="U12" s="5" t="n"/>
+      <c r="V12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1183,6 +1539,10 @@
       <c r="R13" s="5" t="n">
         <v>42000</v>
       </c>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="5" t="n"/>
+      <c r="V13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1229,6 +1589,10 @@
       <c r="R14" s="5" t="n">
         <v>36000</v>
       </c>
+      <c r="S14" s="5" t="n"/>
+      <c r="T14" s="5" t="n"/>
+      <c r="U14" s="5" t="n"/>
+      <c r="V14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1275,6 +1639,10 @@
       <c r="R15" s="5" t="n">
         <v>25000</v>
       </c>
+      <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="5" t="n"/>
+      <c r="V15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1318,6 +1686,10 @@
       <c r="O16" s="6" t="n"/>
       <c r="P16" s="6" t="n"/>
       <c r="Q16" s="6" t="n"/>
+      <c r="S16" s="5" t="n"/>
+      <c r="T16" s="5" t="n"/>
+      <c r="U16" s="5" t="n"/>
+      <c r="V16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1364,6 +1736,10 @@
       <c r="R17" s="5" t="n">
         <v>60000</v>
       </c>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="U17" s="5" t="n"/>
+      <c r="V17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1410,6 +1786,10 @@
       <c r="R18" s="5" t="n">
         <v>38000</v>
       </c>
+      <c r="S18" s="5" t="n"/>
+      <c r="T18" s="5" t="n"/>
+      <c r="U18" s="5" t="n"/>
+      <c r="V18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1453,6 +1833,10 @@
       <c r="O19" s="6" t="n"/>
       <c r="P19" s="6" t="n"/>
       <c r="Q19" s="6" t="n"/>
+      <c r="S19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
+      <c r="U19" s="5" t="n"/>
+      <c r="V19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1502,6 +1886,10 @@
       <c r="R20" s="5" t="n">
         <v>12000</v>
       </c>
+      <c r="S20" s="5" t="n"/>
+      <c r="T20" s="5" t="n"/>
+      <c r="U20" s="5" t="n"/>
+      <c r="V20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1545,6 +1933,10 @@
       <c r="O21" s="6" t="n"/>
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="6" t="n"/>
+      <c r="S21" s="5" t="n"/>
+      <c r="T21" s="5" t="n"/>
+      <c r="U21" s="5" t="n"/>
+      <c r="V21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1579,6 +1971,10 @@
       <c r="O22" s="6" t="n"/>
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="6" t="n"/>
+      <c r="S22" s="5" t="n"/>
+      <c r="T22" s="5" t="n"/>
+      <c r="U22" s="5" t="n"/>
+      <c r="V22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1613,6 +2009,10 @@
       <c r="O23" s="6" t="n"/>
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="6" t="n"/>
+      <c r="S23" s="5" t="n"/>
+      <c r="T23" s="5" t="n"/>
+      <c r="U23" s="5" t="n"/>
+      <c r="V23" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
V6: rangos por tipo, P10/P90 y aviso de rangos optimistas
- Columnas «P10» y «P90» como alternativa a mínimo y máximo: se calculan
  los extremos de la PERT (o triangular) que dan esos percentiles.
- Chequeo de salud «Rangos realistas» (estrechos, sesgados a acortar,
  todos iguales), también en el oráculo Python («Esperado (salud)»).
- Hoja editable «Rangos por tipo» con valores de partida por tipo de
  trabajo; «Rellenar los rangos vacíos» la usa según categoría o nombre.
- Tests, guía Q53–Q55 y documentación al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -3515,7 +3515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3651,10 +3651,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>optimismo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>convergencias</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>info</t>
         </is>

</xml_diff>

<commit_message>
V7: calendarios por actividad
- Hoja «Calendarios» y columna «Calendario» en «Actividades». Con varios
  calendarios, el CPM y la simulación usan un eje de días naturales y el
  reloj de cada actividad (retardos en el calendario de la predecesora,
  holgura en el de la actividad). Con uno solo, el camino de siempre.
- Importación de calendarios por tarea desde MS Project (XML) y P6 (XER).
- En la simulación, las restricciones tardías se aplican dentro de la
  pasada atrás, como en el CPM determinista.
- Oráculo Python con relojes («Calendarios (prueba)», «Esperado
  (calendarios)»); pruebas de equivalencia y en varios hilos; benchmark
  con calendarios; guía Q56–Q58.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -18,6 +18,8 @@
     <sheet name="Esperado (con avance)" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Costos inciertos (prueba)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Esperado (costos inciertos)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Calendarios (prueba)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Esperado (calendarios)" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -578,55 +580,69 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>«Calendarios (prueba)» y «Esperado (calendarios)»: tres calendarios (6 días, continuo, proveedor</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>extranjero) para cuatro actividades, con su CPM y su Monte Carlo de referencia (V7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Cómo se usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>bloque Q (docs/GUIA_PRUEBAS_EXCEL.md).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Resultado esperado, en una línea</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Fin del proyecto: 16/07/2027 · 118 días laborables · 12 actividades críticas.</t>
         </is>
@@ -917,13 +933,1466 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>V7: copia la tabla de abajo en una hoja nueva «Calendarios» (desde A3) y escribe el calendario de cada actividad en la columna «Calendario» de «Actividades» (las demás, vacías: calendario del proyecto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Festivos del proyecto</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Festivos propios (dd/mm/aaaa; …)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>6 días</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Continuo</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>31/05/2027; 05/07/2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Calendario</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>6 días</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6 días</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Proveedor</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Continuo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="3" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>CPM esperado con «Calendarios (prueba)», calculado por el script: eje de días naturales; retardos en el calendario de la predecesora; holgura en días del calendario de cada actividad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fin del proyecto</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46582</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Duración (días naturales)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Duración</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Fin</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Inicio tardío</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Fin tardío</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Holgura total</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Crítica</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Monte Carlo (Python)</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inicio del proyecto</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>46425</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>46425</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>46584</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>1246726.33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Permisos y licencias</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>46437</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>46426</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>46601</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>1293581.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Diseño detallado</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>46419</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>46426</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>46451</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>P80</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>46611</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>1328784.99</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Movilización de obra</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>46440</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>46444</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>46451</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>46618</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>1348637.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Excavación</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>46447</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>46458</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>46454</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>46465</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>JCL</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.7596000000000001</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cimentación</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>46459</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>46478</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>46466</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>46485</v>
+      </c>
+      <c r="H11" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Estructura</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>46479</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>46514</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>46486</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>46521</v>
+      </c>
+      <c r="H12" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Criticidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fabricación del ascensor</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>45</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>46454</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>46514</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>46504</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>46567</v>
+      </c>
+      <c r="H13" t="n">
+        <v>36</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>0.768</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cubierta</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>46517</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>46532</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>46527</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>46542</v>
+      </c>
+      <c r="H14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0.579</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>46491</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>46518</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>46517</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>46542</v>
+      </c>
+      <c r="H15" t="n">
+        <v>18</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>0.189</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Instalaciones hidráulicas</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>18</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>46491</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>46514</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>46519</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>46542</v>
+      </c>
+      <c r="H16" t="n">
+        <v>20</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0.579</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mampostería</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>46510</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>46535</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>46517</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>46542</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>0.767</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Montaje del ascensor</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>46533</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>46542</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>46568</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>46577</v>
+      </c>
+      <c r="H18" t="n">
+        <v>25</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0.767</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Acabados interiores</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>25</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>46538</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>46570</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>46545</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>46577</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>0.767</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Fachada</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>15</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>46533</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>46553</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>46545</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>46563</v>
+      </c>
+      <c r="H20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Pruebas de instalaciones</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>46514</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>46521</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>46570</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>46577</v>
+      </c>
+      <c r="H21" t="n">
+        <v>40</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>0.061</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Paisajismo</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>46566</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>46577</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>46566</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>46577</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Limpieza final</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>46580</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>46580</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Entrega al cliente</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Vigilancia hasta la entrega</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>46573</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>46573</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>0.061</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -948,6 +2417,7 @@
     <col width="17" customWidth="1" min="20" max="20"/>
     <col width="19" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1066,6 +2536,11 @@
       <c r="V3" s="3" t="inlineStr">
         <is>
           <t>Costo por día máximo</t>
+        </is>
+      </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>Calendario</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
V10: registro de riesgos completo con matriz de probabilidad e impacto
- «Riesgos de plazo»: categoría, estado, fecha de revisión e impacto
  cualitativo; riesgos solo de costo y cualitativos. Se simulan los
  activos (sin cerrados ni cualitativos; materializados al 100 %).
- evaluarRegistro y hojaRegistro: matriz 5 × 5 con zonas de color, impacto
  del usuario o de la simulación, revisiones vencidas. En el panel, en la
  hoja «Registro de riesgos» y en el informe PDF.
- Corrige que «En seguimiento» no se reconocía como estado.
- Tests y guía Q63–Q64.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -5323,7 +5323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5468,6 +5468,26 @@
           <t>Antes de</t>
         </is>
       </c>
+      <c r="W3" s="3" t="inlineStr">
+        <is>
+          <t>Categoría del riesgo</t>
+        </is>
+      </c>
+      <c r="X3" s="3" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="Y3" s="3" t="inlineStr">
+        <is>
+          <t>Fecha de revisión</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>Impacto cualitativo (1–5)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
W1: hitos contractuales y multas por retraso
- Hoja «Hitos»: fecha contractual, multa por día natural de retraso y
  tope. La simulación da por hito la probabilidad de cumplir, P50/P80,
  margen y multa media; las multas se suman al costo y a la JCL.
- Panel, resumen en palabras, hoja de la simulación e informe PDF.
- Oráculo Python («Hitos (prueba)», «Esperado (hitos)»), caso exacto,
  hilos; guía Q67.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -20,8 +20,10 @@
     <sheet name="Esperado (costos inciertos)" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Calendarios (prueba)" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Esperado (calendarios)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Clima (prueba)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Esperado (clima)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Hitos (prueba)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Esperado (hitos)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Clima (prueba)" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Esperado (clima)" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -610,55 +612,62 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>«Hitos (prueba)» y «Esperado (hitos)»: fechas contractuales y multas por retraso (W1).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Cómo se usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
+          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>bloque Q (docs/GUIA_PRUEBAS_EXCEL.md).</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Resultado esperado, en una línea</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Fin del proyecto: 16/07/2027 · 118 días laborables · 12 actividades críticas.</t>
         </is>
@@ -2408,6 +2417,280 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>W1: copia esta tabla (desde la fila 3) en una hoja «Hitos» (la crea «Plantilla de cronograma»).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Hito (ID)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Fecha contractual</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Multa por día de retraso</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Tope de la multa</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>46612</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Acta de entrega</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>46568</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Puesta en servicio del ascensor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>46528</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Hito de obra (sin multa)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Monte Carlo de referencia con «Hitos (prueba)»: 20000 iteraciones en Python (los mismos números que «Esperado (simulación)»). Probabilidad ±3 puntos, fechas ±1 día, dinero ±2 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Hito</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Probabilidad de cumplir</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>P80</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Multa media</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.6129</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>46610</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>46623</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>9941.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>0.3903</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>46573</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>46582</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3622.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.1168</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>46541</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>46552</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Multas: probabilidad de alguna</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.6212</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Multas: media</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>13564.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Multas: P80</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>29000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Costo P80 (con multas)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1370540.2237</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>JCL (con multas)</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.7792</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2655,7 +2938,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
W5: RIESGO.CRONOGRAMA, el plazo del cronograma en el modelo de costos
La fórmula =RIESGO.CRONOGRAMA(hito; medida; valor_fijo) toma la fecha, los
días, el retraso o la multa de un hito (o el costo del proyecto) en la misma
iteración que los costos: el cronograma del libro se simula con la semilla y
las iteraciones del modelo de costos y sus muestras entran como buffers.
Fuera de la simulación enseña el valor del plan que publica el panel
Cronograma. Contra la referencia en Python («Esperado (costos con plazo)»).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RWU3ynKgtPJTRMrmZJGwfH
</commit_message>
<xml_diff>
--- a/ejemplos/demo-cronograma.xlsx
+++ b/ejemplos/demo-cronograma.xlsx
@@ -22,8 +22,10 @@
     <sheet name="Esperado (calendarios)" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Hitos (prueba)" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Esperado (hitos)" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Clima (prueba)" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Esperado (clima)" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Costos con plazo (prueba)" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Esperado (costos con plazo)" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Clima (prueba)" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Esperado (clima)" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -89,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -101,6 +103,8 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -619,55 +623,69 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>«Costos con plazo (prueba)» y «Esperado (costos con plazo)»: un modelo de costos que toma los días</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>del proyecto y la multa del hito 19 con RIESGO.CRONOGRAMA, en la misma iteración (W5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Cómo se usa</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+          <t>Panel → pestaña Cronograma → «Calcular cronograma». Escribe la hoja «Cronograma (resultado)».</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Compárala con «Esperado»: mismas fechas, misma holgura y mismas actividades críticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Los pasos exactos, y qué tocar para provocar cada error, están en la guía de pruebas,</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>bloque Q (docs/GUIA_PRUEBAS_EXCEL.md).</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Resultado esperado, en una línea</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Fin del proyecto: 16/07/2027 · 118 días laborables · 12 actividades críticas.</t>
         </is>
@@ -2691,6 +2709,222 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>W5: un modelo de costos que toma el plazo del cronograma en la misma iteración. Copia «Hitos (prueba)» como «Hitos», escribe las fórmulas de la columna C en la columna B y marca B8 y B7 como salidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Escribe en la columna B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Obra (sin indirectos)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.TRIANGULAR(900000;1000000;1250000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Días del proyecto</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.CRONOGRAMA("Proyecto";"dias")</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Indirectos (1.500 por día)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>escribe =B4*1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Multa de la entrega (hito 19)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.CRONOGRAMA("19";"multa")</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Fecha de entrega (hito 19)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>escribe =RIESGO.CRONOGRAMA("19";"fecha")</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Costo total</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>escribe =B3+B5+B6+RIESGO.SALIDA("Costo total")</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Referencia en Python de «Costos con plazo (prueba)»: 20000 iteraciones, las mismas del cronograma de «Esperado (hitos)». Dinero ±2 %, fechas ±1 día, probabilidades ±3 puntos, correlación ±0,05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Costo total: media</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1263523.1419</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Costo total: P80</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1334304.031</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fecha de entrega (19): P80</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>46623</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Entrega a tiempo (13/08/2027)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.6129</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Conjunta: costo ≤ P80 y entrega a tiempo</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.5279</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lo mismo si fueran independientes (80 % × a tiempo)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.4903</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Correlación días del proyecto – costo total</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>0.3469</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2938,7 +3172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>